<commit_message>
mofrl fitting for 2010complete birth data file
</commit_message>
<xml_diff>
--- a/model_fitting/2010/model1_ordinal_OR.xlsx
+++ b/model_fitting/2010/model1_ordinal_OR.xlsx
@@ -450,7 +450,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5.6</v>
+        <v>5.601</v>
       </c>
       <c r="C2" t="n">
         <v>5.264</v>
@@ -501,7 +501,7 @@
         <v>44.006</v>
       </c>
       <c r="C4" t="n">
-        <v>41.391</v>
+        <v>41.392</v>
       </c>
       <c r="D4" t="n">
         <v>46.785</v>
@@ -522,13 +522,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>92.51300000000001</v>
+        <v>92.51900000000001</v>
       </c>
       <c r="C5" t="n">
-        <v>86.90600000000001</v>
+        <v>86.913</v>
       </c>
       <c r="D5" t="n">
-        <v>98.48</v>
+        <v>98.488</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -555,7 +555,7 @@
         <v>0.991</v>
       </c>
       <c r="E6" t="n">
-        <v>0.026</v>
+        <v>0.0259</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -573,13 +573,13 @@
         <v>0.583</v>
       </c>
       <c r="C7" t="n">
-        <v>0.219</v>
+        <v>0.226</v>
       </c>
       <c r="D7" t="n">
-        <v>1.554</v>
+        <v>1.506</v>
       </c>
       <c r="E7" t="n">
-        <v>0.2806</v>
+        <v>0.2651</v>
       </c>
       <c r="F7" t="inlineStr"/>
     </row>
@@ -593,13 +593,13 @@
         <v>0.928</v>
       </c>
       <c r="C8" t="n">
-        <v>0.307</v>
+        <v>0.309</v>
       </c>
       <c r="D8" t="n">
-        <v>2.808</v>
+        <v>2.791</v>
       </c>
       <c r="E8" t="n">
-        <v>0.8953</v>
+        <v>0.8947000000000001</v>
       </c>
       <c r="F8" t="inlineStr"/>
     </row>
@@ -613,13 +613,13 @@
         <v>0.988</v>
       </c>
       <c r="C9" t="n">
-        <v>0.378</v>
+        <v>0.39</v>
       </c>
       <c r="D9" t="n">
-        <v>2.581</v>
+        <v>2.501</v>
       </c>
       <c r="E9" t="n">
-        <v>0.9802999999999999</v>
+        <v>0.9797</v>
       </c>
       <c r="F9" t="inlineStr"/>
     </row>
@@ -633,13 +633,13 @@
         <v>0.9350000000000001</v>
       </c>
       <c r="C10" t="n">
-        <v>0.353</v>
+        <v>0.365</v>
       </c>
       <c r="D10" t="n">
-        <v>2.476</v>
+        <v>2.399</v>
       </c>
       <c r="E10" t="n">
-        <v>0.8931</v>
+        <v>0.8895999999999999</v>
       </c>
       <c r="F10" t="inlineStr"/>
     </row>
@@ -653,13 +653,13 @@
         <v>0.351</v>
       </c>
       <c r="C11" t="n">
-        <v>0.126</v>
+        <v>0.13</v>
       </c>
       <c r="D11" t="n">
-        <v>0.977</v>
+        <v>0.948</v>
       </c>
       <c r="E11" t="n">
-        <v>0.045</v>
+        <v>0.0389</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -677,13 +677,13 @@
         <v>0.894</v>
       </c>
       <c r="C12" t="n">
-        <v>0.293</v>
+        <v>0.3</v>
       </c>
       <c r="D12" t="n">
-        <v>2.733</v>
+        <v>2.666</v>
       </c>
       <c r="E12" t="n">
-        <v>0.8447</v>
+        <v>0.8413</v>
       </c>
       <c r="F12" t="inlineStr"/>
     </row>
@@ -697,13 +697,13 @@
         <v>0.542</v>
       </c>
       <c r="C13" t="n">
-        <v>0.193</v>
+        <v>0.198</v>
       </c>
       <c r="D13" t="n">
-        <v>1.525</v>
+        <v>1.484</v>
       </c>
       <c r="E13" t="n">
-        <v>0.2463</v>
+        <v>0.2336</v>
       </c>
       <c r="F13" t="inlineStr"/>
     </row>
@@ -717,13 +717,13 @@
         <v>0.528</v>
       </c>
       <c r="C14" t="n">
-        <v>0.202</v>
+        <v>0.209</v>
       </c>
       <c r="D14" t="n">
-        <v>1.378</v>
+        <v>1.336</v>
       </c>
       <c r="E14" t="n">
-        <v>0.192</v>
+        <v>0.1774</v>
       </c>
       <c r="F14" t="inlineStr"/>
     </row>
@@ -737,13 +737,13 @@
         <v>0.9419999999999999</v>
       </c>
       <c r="C15" t="n">
-        <v>0.163</v>
+        <v>0.173</v>
       </c>
       <c r="D15" t="n">
-        <v>5.431</v>
+        <v>5.132</v>
       </c>
       <c r="E15" t="n">
-        <v>0.9463</v>
+        <v>0.9445</v>
       </c>
       <c r="F15" t="inlineStr"/>
     </row>
@@ -757,13 +757,13 @@
         <v>1.283</v>
       </c>
       <c r="C16" t="n">
-        <v>0.491</v>
+        <v>0.507</v>
       </c>
       <c r="D16" t="n">
-        <v>3.351</v>
+        <v>3.247</v>
       </c>
       <c r="E16" t="n">
-        <v>0.6105</v>
+        <v>0.5984</v>
       </c>
       <c r="F16" t="inlineStr"/>
     </row>
@@ -777,13 +777,13 @@
         <v>0.895</v>
       </c>
       <c r="C17" t="n">
-        <v>0.343</v>
+        <v>0.354</v>
       </c>
       <c r="D17" t="n">
-        <v>2.337</v>
+        <v>2.264</v>
       </c>
       <c r="E17" t="n">
-        <v>0.8204</v>
+        <v>0.8145</v>
       </c>
       <c r="F17" t="inlineStr"/>
     </row>
@@ -848,10 +848,10 @@
         <v>0.582</v>
       </c>
       <c r="D20" t="n">
-        <v>1.83</v>
+        <v>1.829</v>
       </c>
       <c r="E20" t="n">
-        <v>0.915</v>
+        <v>0.9149</v>
       </c>
       <c r="F20" t="inlineStr"/>
     </row>

</xml_diff>